<commit_message>
feat(orcamento): abas de apoio com as contas pagas do financeiro
Extrato de 419 lancamentos de jan a jul/26 entra como duas abas por
planilha, separadas pelo centro de custo que o proprio extrato ja traz
("Juridico" 319 lanc. / "T.I" 100 lanc.):

- Contas Pagas (resumo): por credor, com os valores mes a mes
- Contas Pagas (detalhe): um lancamento por linha, com filtro

Sao abas de APOIO e nada delas alimenta o Planejado, o Realizado ou o
Painel — o centro de custo desses itens ainda sera decidido com a
diretoria, e misturar agora contaminaria o comparativo.

A ultima coluna do resumo aponta, por palavra-chave no nome do credor,
qual linha do orcamento aquele pagamento provavelmente duplica, com a
linha inteira destacada em amarelo. Serve para a remocao manual das
duplicidades.

Arquivo de origem versionado em dados/ para a geracao ser reproduzivel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wiPdT7yF96oyPU7xT24sa
</commit_message>
<xml_diff>
--- a/orcamento/Orcamento_TI_2026.xlsx
+++ b/orcamento/Orcamento_TI_2026.xlsx
@@ -15,10 +15,14 @@
     <sheet name="Por Plano de Contas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Pendências" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Como usar" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Contas Pagas (resumo)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Contas Pagas (detalhe)" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Comparativo'!$A$5:$N$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Planejado'!$A$4:$T$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Contas Pagas (resumo)'!$A$4:$L$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Contas Pagas (detalhe)'!$A$4:$H$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +34,7 @@
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -138,10 +142,15 @@
       <sz val="9"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="8"/>
+    </font>
+    <font>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -213,6 +222,11 @@
         <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -240,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -396,9 +410,26 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1820,6 +1851,4054 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H105"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTAS PAGAS — DETALHE  (TI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Um lançamento por linha, como veio do financeiro. Use o filtro do cabeçalho para conferir credor, empreendimento ou mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>Mês</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Data de Pagamento</t>
+        </is>
+      </c>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>Credor</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
+        <is>
+          <t>Documento</t>
+        </is>
+      </c>
+      <c r="E4" s="46" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="F4" s="46" t="inlineStr">
+        <is>
+          <t>Empreendimento</t>
+        </is>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>Valor Líquido</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B5" s="79" t="inlineStr">
+        <is>
+          <t>09/01/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D5" s="79" t="inlineStr">
+        <is>
+          <t>FAT.11.25</t>
+        </is>
+      </c>
+      <c r="E5" s="79" t="inlineStr">
+        <is>
+          <t>95941/1</t>
+        </is>
+      </c>
+      <c r="F5" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G5" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H5" s="80" t="n">
+        <v>407.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B6" s="79" t="inlineStr">
+        <is>
+          <t>28/01/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D6" s="79" t="inlineStr">
+        <is>
+          <t>FAT.01.26</t>
+        </is>
+      </c>
+      <c r="E6" s="79" t="inlineStr">
+        <is>
+          <t>97478/1</t>
+        </is>
+      </c>
+      <c r="F6" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G6" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H6" s="80" t="n">
+        <v>390.95</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B7" s="79" t="inlineStr">
+        <is>
+          <t>28/01/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D7" s="79" t="inlineStr">
+        <is>
+          <t>FAT.184180933</t>
+        </is>
+      </c>
+      <c r="E7" s="79" t="inlineStr">
+        <is>
+          <t>97480/1</t>
+        </is>
+      </c>
+      <c r="F7" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G7" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H7" s="80" t="n">
+        <v>123.76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B8" s="79" t="inlineStr">
+        <is>
+          <t>30/01/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D8" s="79" t="inlineStr">
+        <is>
+          <t>NFS.347106</t>
+        </is>
+      </c>
+      <c r="E8" s="79" t="inlineStr">
+        <is>
+          <t>96534/1</t>
+        </is>
+      </c>
+      <c r="F8" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G8" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H8" s="80" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B9" s="79" t="inlineStr">
+        <is>
+          <t>19/01/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="79" t="inlineStr">
+        <is>
+          <t>J H ALVES - MONITOR REMOTO</t>
+        </is>
+      </c>
+      <c r="D9" s="79" t="inlineStr">
+        <is>
+          <t>NFS.70</t>
+        </is>
+      </c>
+      <c r="E9" s="79" t="inlineStr">
+        <is>
+          <t>96602/1</t>
+        </is>
+      </c>
+      <c r="F9" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G9" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H9" s="80" t="n">
+        <v>4311.56</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B10" s="79" t="inlineStr">
+        <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D10" s="79" t="inlineStr">
+        <is>
+          <t>AV.LIC EMAILS 01.25</t>
+        </is>
+      </c>
+      <c r="E10" s="79" t="inlineStr">
+        <is>
+          <t>96014/1</t>
+        </is>
+      </c>
+      <c r="F10" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G10" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H10" s="80" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B11" s="79" t="inlineStr">
+        <is>
+          <t>25/01/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D11" s="79" t="inlineStr">
+        <is>
+          <t>BOL.13.01</t>
+        </is>
+      </c>
+      <c r="E11" s="79" t="inlineStr">
+        <is>
+          <t>96623/1</t>
+        </is>
+      </c>
+      <c r="F11" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G11" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H11" s="80" t="n">
+        <v>918.08</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B12" s="79" t="inlineStr">
+        <is>
+          <t>30/01/2026</t>
+        </is>
+      </c>
+      <c r="C12" s="79" t="inlineStr">
+        <is>
+          <t>SABHA INTELIGENCIA EM TECNOLOGIA LTDA</t>
+        </is>
+      </c>
+      <c r="D12" s="79" t="inlineStr">
+        <is>
+          <t>FAT.2682</t>
+        </is>
+      </c>
+      <c r="E12" s="79" t="inlineStr">
+        <is>
+          <t>96458/1</t>
+        </is>
+      </c>
+      <c r="F12" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G12" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H12" s="80" t="n">
+        <v>723.75</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B13" s="79" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D13" s="79" t="inlineStr">
+        <is>
+          <t>FAT.2011241340</t>
+        </is>
+      </c>
+      <c r="E13" s="79" t="inlineStr">
+        <is>
+          <t>96088/1</t>
+        </is>
+      </c>
+      <c r="F13" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G13" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H13" s="80" t="n">
+        <v>51.63</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B14" s="79" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="C14" s="79" t="inlineStr">
+        <is>
+          <t>TIM S A</t>
+        </is>
+      </c>
+      <c r="D14" s="79" t="inlineStr">
+        <is>
+          <t>FAT.5664047504</t>
+        </is>
+      </c>
+      <c r="E14" s="79" t="inlineStr">
+        <is>
+          <t>96789/1</t>
+        </is>
+      </c>
+      <c r="F14" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G14" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H14" s="80" t="n">
+        <v>331.42</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B15" s="79" t="inlineStr">
+        <is>
+          <t>26/01/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D15" s="79" t="inlineStr">
+        <is>
+          <t>CX.16.01.26</t>
+        </is>
+      </c>
+      <c r="E15" s="79" t="inlineStr">
+        <is>
+          <t>97067/1</t>
+        </is>
+      </c>
+      <c r="F15" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G15" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H15" s="80" t="n">
+        <v>39.84</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B16" s="79" t="inlineStr">
+        <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D16" s="79" t="inlineStr">
+        <is>
+          <t>SAL.Sal_122025</t>
+        </is>
+      </c>
+      <c r="E16" s="79" t="inlineStr">
+        <is>
+          <t>96252/1</t>
+        </is>
+      </c>
+      <c r="F16" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G16" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H16" s="80" t="n">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B17" s="79" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="C17" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D17" s="79" t="inlineStr">
+        <is>
+          <t>SAL.VALE_ 012026</t>
+        </is>
+      </c>
+      <c r="E17" s="79" t="inlineStr">
+        <is>
+          <t>97269/1</t>
+        </is>
+      </c>
+      <c r="F17" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G17" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H17" s="80" t="n">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="79" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="B18" s="79" t="inlineStr">
+        <is>
+          <t>27/01/2026</t>
+        </is>
+      </c>
+      <c r="C18" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D18" s="79" t="inlineStr">
+        <is>
+          <t>BOL.1</t>
+        </is>
+      </c>
+      <c r="E18" s="79" t="inlineStr">
+        <is>
+          <t>97204/1</t>
+        </is>
+      </c>
+      <c r="F18" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G18" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H18" s="80" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B19" s="79" t="inlineStr">
+        <is>
+          <t>04/02/2026</t>
+        </is>
+      </c>
+      <c r="C19" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D19" s="79" t="inlineStr">
+        <is>
+          <t>AV.04.02.26</t>
+        </is>
+      </c>
+      <c r="E19" s="79" t="inlineStr">
+        <is>
+          <t>98500/1</t>
+        </is>
+      </c>
+      <c r="F19" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G19" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H19" s="80" t="n">
+        <v>26.67</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B20" s="79" t="inlineStr">
+        <is>
+          <t>15/02/2026</t>
+        </is>
+      </c>
+      <c r="C20" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D20" s="79" t="inlineStr">
+        <is>
+          <t>AV.12.02.26 LCW</t>
+        </is>
+      </c>
+      <c r="E20" s="79" t="inlineStr">
+        <is>
+          <t>99336/1</t>
+        </is>
+      </c>
+      <c r="F20" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G20" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H20" s="80" t="n">
+        <v>72.58</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B21" s="79" t="inlineStr">
+        <is>
+          <t>15/02/2026</t>
+        </is>
+      </c>
+      <c r="C21" s="79" t="inlineStr">
+        <is>
+          <t>OPENAI BRAZIL LIMITADA</t>
+        </is>
+      </c>
+      <c r="D21" s="79" t="inlineStr">
+        <is>
+          <t>AV.CHATGPT JUR 2026</t>
+        </is>
+      </c>
+      <c r="E21" s="79" t="inlineStr">
+        <is>
+          <t>95104/2</t>
+        </is>
+      </c>
+      <c r="F21" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G21" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H21" s="80" t="n">
+        <v>234.46</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B22" s="79" t="inlineStr">
+        <is>
+          <t>24/02/2026</t>
+        </is>
+      </c>
+      <c r="C22" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D22" s="79" t="inlineStr">
+        <is>
+          <t>FAT.3575377</t>
+        </is>
+      </c>
+      <c r="E22" s="79" t="inlineStr">
+        <is>
+          <t>100172/1</t>
+        </is>
+      </c>
+      <c r="F22" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G22" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H22" s="80" t="n">
+        <v>52.32</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B23" s="79" t="inlineStr">
+        <is>
+          <t>24/02/2026</t>
+        </is>
+      </c>
+      <c r="C23" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D23" s="79" t="inlineStr">
+        <is>
+          <t>FAT.5290953</t>
+        </is>
+      </c>
+      <c r="E23" s="79" t="inlineStr">
+        <is>
+          <t>100173/1</t>
+        </is>
+      </c>
+      <c r="F23" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G23" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H23" s="80" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B24" s="79" t="inlineStr">
+        <is>
+          <t>27/02/2026</t>
+        </is>
+      </c>
+      <c r="C24" s="79" t="inlineStr">
+        <is>
+          <t>TIM S A</t>
+        </is>
+      </c>
+      <c r="D24" s="79" t="inlineStr">
+        <is>
+          <t>BOL.141</t>
+        </is>
+      </c>
+      <c r="E24" s="79" t="inlineStr">
+        <is>
+          <t>99947/1</t>
+        </is>
+      </c>
+      <c r="F24" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G24" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H24" s="80" t="n">
+        <v>338.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B25" s="79" t="inlineStr">
+        <is>
+          <t>13/02/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="79" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="D25" s="79" t="inlineStr">
+        <is>
+          <t>BOL.26449</t>
+        </is>
+      </c>
+      <c r="E25" s="79" t="inlineStr">
+        <is>
+          <t>99484/1</t>
+        </is>
+      </c>
+      <c r="F25" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G25" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H25" s="80" t="n">
+        <v>137.94</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B26" s="79" t="inlineStr">
+        <is>
+          <t>19/02/2026</t>
+        </is>
+      </c>
+      <c r="C26" s="79" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="D26" s="79" t="inlineStr">
+        <is>
+          <t>BOL.27256</t>
+        </is>
+      </c>
+      <c r="E26" s="79" t="inlineStr">
+        <is>
+          <t>99486/1</t>
+        </is>
+      </c>
+      <c r="F26" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G26" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H26" s="80" t="n">
+        <v>137.9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B27" s="79" t="inlineStr">
+        <is>
+          <t>06/02/2026</t>
+        </is>
+      </c>
+      <c r="C27" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D27" s="79" t="inlineStr">
+        <is>
+          <t>SAL.SAL JANEIRO 2026</t>
+        </is>
+      </c>
+      <c r="E27" s="79" t="inlineStr">
+        <is>
+          <t>98811/1</t>
+        </is>
+      </c>
+      <c r="F27" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G27" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H27" s="80" t="n">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B28" s="79" t="inlineStr">
+        <is>
+          <t>20/02/2026</t>
+        </is>
+      </c>
+      <c r="C28" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D28" s="79" t="inlineStr">
+        <is>
+          <t>SAL.VALE FEVEREIRO 26</t>
+        </is>
+      </c>
+      <c r="E28" s="79" t="inlineStr">
+        <is>
+          <t>99890/1</t>
+        </is>
+      </c>
+      <c r="F28" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G28" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H28" s="80" t="n">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B29" s="79" t="inlineStr">
+        <is>
+          <t>2026-02-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="C29" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D29" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E29" s="79" t="inlineStr">
+        <is>
+          <t>113754/2</t>
+        </is>
+      </c>
+      <c r="F29" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G29" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H29" s="80" t="n">
+        <v>207.04</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B30" s="79" t="inlineStr">
+        <is>
+          <t>2026-02-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="C30" s="79" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="D30" s="79" t="inlineStr"/>
+      <c r="E30" s="79" t="inlineStr"/>
+      <c r="F30" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G30" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H30" s="80" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="79" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="B31" s="79" t="inlineStr">
+        <is>
+          <t>27/02/2026</t>
+        </is>
+      </c>
+      <c r="C31" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D31" s="79" t="inlineStr">
+        <is>
+          <t>NFS.1430</t>
+        </is>
+      </c>
+      <c r="E31" s="79" t="inlineStr">
+        <is>
+          <t>99956/1</t>
+        </is>
+      </c>
+      <c r="F31" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G31" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H31" s="80" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B32" s="79" t="inlineStr">
+        <is>
+          <t>05/03/2026</t>
+        </is>
+      </c>
+      <c r="C32" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D32" s="79" t="inlineStr">
+        <is>
+          <t>FAT.5042829</t>
+        </is>
+      </c>
+      <c r="E32" s="79" t="inlineStr">
+        <is>
+          <t>100503/1</t>
+        </is>
+      </c>
+      <c r="F32" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G32" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H32" s="80" t="n">
+        <v>87.69</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B33" s="79" t="inlineStr">
+        <is>
+          <t>05/03/2026</t>
+        </is>
+      </c>
+      <c r="C33" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D33" s="79" t="inlineStr">
+        <is>
+          <t>FAT.5042827</t>
+        </is>
+      </c>
+      <c r="E33" s="79" t="inlineStr">
+        <is>
+          <t>100504/1</t>
+        </is>
+      </c>
+      <c r="F33" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G33" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H33" s="80" t="n">
+        <v>382.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B34" s="79" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="C34" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D34" s="79" t="inlineStr">
+        <is>
+          <t>FAT.8910508</t>
+        </is>
+      </c>
+      <c r="E34" s="79" t="inlineStr">
+        <is>
+          <t>102706/1</t>
+        </is>
+      </c>
+      <c r="F34" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G34" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H34" s="80" t="n">
+        <v>429.49</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B35" s="79" t="inlineStr">
+        <is>
+          <t>02/03/2026</t>
+        </is>
+      </c>
+      <c r="C35" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D35" s="79" t="inlineStr">
+        <is>
+          <t>NFS.351653</t>
+        </is>
+      </c>
+      <c r="E35" s="79" t="inlineStr">
+        <is>
+          <t>100083/1</t>
+        </is>
+      </c>
+      <c r="F35" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G35" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H35" s="80" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B36" s="79" t="inlineStr">
+        <is>
+          <t>30/03/2026</t>
+        </is>
+      </c>
+      <c r="C36" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D36" s="79" t="inlineStr">
+        <is>
+          <t>NFS.359396</t>
+        </is>
+      </c>
+      <c r="E36" s="79" t="inlineStr">
+        <is>
+          <t>102608/1</t>
+        </is>
+      </c>
+      <c r="F36" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G36" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H36" s="80" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B37" s="79" t="inlineStr">
+        <is>
+          <t>01/03/2026</t>
+        </is>
+      </c>
+      <c r="C37" s="79" t="inlineStr">
+        <is>
+          <t>OPENAI BRAZIL LIMITADA</t>
+        </is>
+      </c>
+      <c r="D37" s="79" t="inlineStr">
+        <is>
+          <t>AV.CHATGPT JUR 2026</t>
+        </is>
+      </c>
+      <c r="E37" s="79" t="inlineStr">
+        <is>
+          <t>95104/3</t>
+        </is>
+      </c>
+      <c r="F37" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G37" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H37" s="80" t="n">
+        <v>111.38</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B38" s="79" t="inlineStr">
+        <is>
+          <t>31/03/2026</t>
+        </is>
+      </c>
+      <c r="C38" s="79" t="inlineStr">
+        <is>
+          <t>OPENAI BRAZIL LIMITADA</t>
+        </is>
+      </c>
+      <c r="D38" s="79" t="inlineStr">
+        <is>
+          <t>AV.CHATGPT JUR 2026</t>
+        </is>
+      </c>
+      <c r="E38" s="79" t="inlineStr">
+        <is>
+          <t>95104/4</t>
+        </is>
+      </c>
+      <c r="F38" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G38" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H38" s="80" t="n">
+        <v>210.38</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B39" s="79" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="C39" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D39" s="79" t="inlineStr">
+        <is>
+          <t>FAT.2024588614</t>
+        </is>
+      </c>
+      <c r="E39" s="79" t="inlineStr">
+        <is>
+          <t>102316/1</t>
+        </is>
+      </c>
+      <c r="F39" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G39" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H39" s="80" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B40" s="79" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="C40" s="79" t="inlineStr">
+        <is>
+          <t>TIM S A</t>
+        </is>
+      </c>
+      <c r="D40" s="79" t="inlineStr">
+        <is>
+          <t>BOL.5708173302</t>
+        </is>
+      </c>
+      <c r="E40" s="79" t="inlineStr">
+        <is>
+          <t>102057/1</t>
+        </is>
+      </c>
+      <c r="F40" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G40" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H40" s="80" t="n">
+        <v>284.63</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B41" s="79" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="C41" s="79" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="D41" s="79" t="inlineStr">
+        <is>
+          <t>BOL.28049</t>
+        </is>
+      </c>
+      <c r="E41" s="79" t="inlineStr">
+        <is>
+          <t>100887/1</t>
+        </is>
+      </c>
+      <c r="F41" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G41" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H41" s="80" t="n">
+        <v>137.9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B42" s="79" t="inlineStr">
+        <is>
+          <t>06/03/2026</t>
+        </is>
+      </c>
+      <c r="C42" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D42" s="79" t="inlineStr">
+        <is>
+          <t>SAL.SAL FEVEREIRO 26</t>
+        </is>
+      </c>
+      <c r="E42" s="79" t="inlineStr">
+        <is>
+          <t>101276/1</t>
+        </is>
+      </c>
+      <c r="F42" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G42" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H42" s="80" t="n">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B43" s="79" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="C43" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D43" s="79" t="inlineStr">
+        <is>
+          <t>SAL.VALE 032026</t>
+        </is>
+      </c>
+      <c r="E43" s="79" t="inlineStr">
+        <is>
+          <t>102295/1</t>
+        </is>
+      </c>
+      <c r="F43" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G43" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H43" s="80" t="n">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B44" s="79" t="inlineStr">
+        <is>
+          <t>2026-03-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="C44" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D44" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E44" s="79" t="inlineStr">
+        <is>
+          <t>113754/3</t>
+        </is>
+      </c>
+      <c r="F44" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G44" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H44" s="80" t="n">
+        <v>207.04</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B45" s="79" t="inlineStr">
+        <is>
+          <t>2026-03-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="C45" s="79" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="D45" s="79" t="inlineStr"/>
+      <c r="E45" s="79" t="inlineStr"/>
+      <c r="F45" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G45" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H45" s="80" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B46" s="79" t="inlineStr">
+        <is>
+          <t>25/03/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D46" s="79" t="inlineStr">
+        <is>
+          <t>NFS.1500</t>
+        </is>
+      </c>
+      <c r="E46" s="79" t="inlineStr">
+        <is>
+          <t>102432/1</t>
+        </is>
+      </c>
+      <c r="F46" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G46" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H46" s="80" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="79" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="B47" s="79" t="inlineStr">
+        <is>
+          <t>25/03/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D47" s="79" t="inlineStr">
+        <is>
+          <t>NFS.1534</t>
+        </is>
+      </c>
+      <c r="E47" s="79" t="inlineStr">
+        <is>
+          <t>102434/1</t>
+        </is>
+      </c>
+      <c r="F47" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G47" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H47" s="80" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B48" s="79" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D48" s="79" t="inlineStr">
+        <is>
+          <t>FAT.8910315</t>
+        </is>
+      </c>
+      <c r="E48" s="79" t="inlineStr">
+        <is>
+          <t>105607/1</t>
+        </is>
+      </c>
+      <c r="F48" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G48" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H48" s="80" t="n">
+        <v>11.99</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B49" s="79" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D49" s="79" t="inlineStr">
+        <is>
+          <t>FAT.13443658</t>
+        </is>
+      </c>
+      <c r="E49" s="79" t="inlineStr">
+        <is>
+          <t>105676/1</t>
+        </is>
+      </c>
+      <c r="F49" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G49" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H49" s="80" t="n">
+        <v>557.63</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B50" s="79" t="inlineStr">
+        <is>
+          <t>29/04/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D50" s="79" t="inlineStr">
+        <is>
+          <t>FAT.13443664</t>
+        </is>
+      </c>
+      <c r="E50" s="79" t="inlineStr">
+        <is>
+          <t>105677/1</t>
+        </is>
+      </c>
+      <c r="F50" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G50" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H50" s="80" t="n">
+        <v>132.09</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B51" s="79" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D51" s="79" t="inlineStr">
+        <is>
+          <t>FAT.13443112</t>
+        </is>
+      </c>
+      <c r="E51" s="79" t="inlineStr">
+        <is>
+          <t>105792/1</t>
+        </is>
+      </c>
+      <c r="F51" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G51" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H51" s="80" t="n">
+        <v>20.23</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B52" s="79" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="C52" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D52" s="79" t="inlineStr">
+        <is>
+          <t>NFS.363799</t>
+        </is>
+      </c>
+      <c r="E52" s="79" t="inlineStr">
+        <is>
+          <t>104634/1</t>
+        </is>
+      </c>
+      <c r="F52" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G52" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H52" s="80" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B53" s="79" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="C53" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D53" s="79" t="inlineStr">
+        <is>
+          <t>BOL.04.26</t>
+        </is>
+      </c>
+      <c r="E53" s="79" t="inlineStr">
+        <is>
+          <t>104820/1</t>
+        </is>
+      </c>
+      <c r="F53" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G53" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H53" s="80" t="n">
+        <v>1024.76</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B54" s="79" t="inlineStr">
+        <is>
+          <t>30/04/2026</t>
+        </is>
+      </c>
+      <c r="C54" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D54" s="79" t="inlineStr">
+        <is>
+          <t>BOL.LOCAWEB 29.04.26</t>
+        </is>
+      </c>
+      <c r="E54" s="79" t="inlineStr">
+        <is>
+          <t>106325/1</t>
+        </is>
+      </c>
+      <c r="F54" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G54" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H54" s="80" t="n">
+        <v>21.76</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B55" s="79" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="C55" s="79" t="inlineStr">
+        <is>
+          <t>OPENAI BRAZIL LIMITADA</t>
+        </is>
+      </c>
+      <c r="D55" s="79" t="inlineStr">
+        <is>
+          <t>FAT.CHATGPT 3 LIC</t>
+        </is>
+      </c>
+      <c r="E55" s="79" t="inlineStr">
+        <is>
+          <t>102137/1</t>
+        </is>
+      </c>
+      <c r="F55" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G55" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H55" s="80" t="n">
+        <v>5393.88</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B56" s="79" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="C56" s="79" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="D56" s="79" t="inlineStr">
+        <is>
+          <t>BOL.28855</t>
+        </is>
+      </c>
+      <c r="E56" s="79" t="inlineStr">
+        <is>
+          <t>103694/1</t>
+        </is>
+      </c>
+      <c r="F56" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G56" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H56" s="80" t="n">
+        <v>137.9</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B57" s="79" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C57" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D57" s="79" t="inlineStr">
+        <is>
+          <t>SAL.SAL 032026</t>
+        </is>
+      </c>
+      <c r="E57" s="79" t="inlineStr">
+        <is>
+          <t>103924/1</t>
+        </is>
+      </c>
+      <c r="F57" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G57" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H57" s="80" t="n">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B58" s="79" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="C58" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D58" s="79" t="inlineStr">
+        <is>
+          <t>SAL.vale 042026</t>
+        </is>
+      </c>
+      <c r="E58" s="79" t="inlineStr">
+        <is>
+          <t>105055/1</t>
+        </is>
+      </c>
+      <c r="F58" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G58" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H58" s="80" t="n">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B59" s="79" t="inlineStr">
+        <is>
+          <t>2026-04-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="C59" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D59" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E59" s="79" t="inlineStr">
+        <is>
+          <t>113754/4</t>
+        </is>
+      </c>
+      <c r="F59" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G59" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H59" s="80" t="n">
+        <v>207.04</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B60" s="79" t="inlineStr">
+        <is>
+          <t>2026-04-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="C60" s="79" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="D60" s="79" t="inlineStr"/>
+      <c r="E60" s="79" t="inlineStr"/>
+      <c r="F60" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G60" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H60" s="80" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="79" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="B61" s="79" t="inlineStr">
+        <is>
+          <t>27/04/2026</t>
+        </is>
+      </c>
+      <c r="C61" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D61" s="79" t="inlineStr">
+        <is>
+          <t>NFS.1573</t>
+        </is>
+      </c>
+      <c r="E61" s="79" t="inlineStr">
+        <is>
+          <t>105411/1</t>
+        </is>
+      </c>
+      <c r="F61" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G61" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H61" s="80" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B62" s="79" t="inlineStr">
+        <is>
+          <t>18/05/2026</t>
+        </is>
+      </c>
+      <c r="C62" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D62" s="79" t="inlineStr">
+        <is>
+          <t>FAT.2ªvia Claro Abril</t>
+        </is>
+      </c>
+      <c r="E62" s="79" t="inlineStr">
+        <is>
+          <t>107340/1</t>
+        </is>
+      </c>
+      <c r="F62" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G62" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H62" s="80" t="n">
+        <v>182.32</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B63" s="79" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="C63" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D63" s="79" t="inlineStr">
+        <is>
+          <t>FAT.17483469</t>
+        </is>
+      </c>
+      <c r="E63" s="79" t="inlineStr">
+        <is>
+          <t>108218/1</t>
+        </is>
+      </c>
+      <c r="F63" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G63" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H63" s="80" t="n">
+        <v>629.98</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B64" s="79" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="C64" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D64" s="79" t="inlineStr">
+        <is>
+          <t>FAT.17483469</t>
+        </is>
+      </c>
+      <c r="E64" s="79" t="inlineStr">
+        <is>
+          <t>108218/2</t>
+        </is>
+      </c>
+      <c r="F64" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G64" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H64" s="80" t="n">
+        <v>18.86</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B65" s="79" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="C65" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D65" s="79" t="inlineStr">
+        <is>
+          <t>FAT.17483469</t>
+        </is>
+      </c>
+      <c r="E65" s="79" t="inlineStr">
+        <is>
+          <t>108218/3</t>
+        </is>
+      </c>
+      <c r="F65" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G65" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H65" s="80" t="n">
+        <v>133.95</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B66" s="79" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="C66" s="79" t="inlineStr">
+        <is>
+          <t>J H ALVES - MONITOR REMOTO</t>
+        </is>
+      </c>
+      <c r="D66" s="79" t="inlineStr">
+        <is>
+          <t>NFS.76</t>
+        </is>
+      </c>
+      <c r="E66" s="79" t="inlineStr">
+        <is>
+          <t>105987/1</t>
+        </is>
+      </c>
+      <c r="F66" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G66" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H66" s="80" t="n">
+        <v>3723.62</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B67" s="79" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="C67" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D67" s="79" t="inlineStr">
+        <is>
+          <t>BOL.LOCAWEB 11.05.26</t>
+        </is>
+      </c>
+      <c r="E67" s="79" t="inlineStr">
+        <is>
+          <t>107254/1</t>
+        </is>
+      </c>
+      <c r="F67" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G67" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H67" s="80" t="n">
+        <v>74.81</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B68" s="79" t="inlineStr">
+        <is>
+          <t>12/05/2026</t>
+        </is>
+      </c>
+      <c r="C68" s="79" t="inlineStr">
+        <is>
+          <t>SABHA INTELIGENCIA EM TECNOLOGIA LTDA</t>
+        </is>
+      </c>
+      <c r="D68" s="79" t="inlineStr">
+        <is>
+          <t>NFS.5744</t>
+        </is>
+      </c>
+      <c r="E68" s="79" t="inlineStr">
+        <is>
+          <t>106664/1</t>
+        </is>
+      </c>
+      <c r="F68" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G68" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H68" s="80" t="n">
+        <v>741.1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B69" s="79" t="inlineStr">
+        <is>
+          <t>25/05/2026</t>
+        </is>
+      </c>
+      <c r="C69" s="79" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="D69" s="79" t="inlineStr">
+        <is>
+          <t>BOL.29637</t>
+        </is>
+      </c>
+      <c r="E69" s="79" t="inlineStr">
+        <is>
+          <t>108040/1</t>
+        </is>
+      </c>
+      <c r="F69" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G69" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H69" s="80" t="n">
+        <v>137.92</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B70" s="79" t="inlineStr">
+        <is>
+          <t>07/05/2026</t>
+        </is>
+      </c>
+      <c r="C70" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D70" s="79" t="inlineStr">
+        <is>
+          <t>SAL.sal 042026</t>
+        </is>
+      </c>
+      <c r="E70" s="79" t="inlineStr">
+        <is>
+          <t>106947/1</t>
+        </is>
+      </c>
+      <c r="F70" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G70" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H70" s="80" t="n">
+        <v>1483</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B71" s="79" t="inlineStr">
+        <is>
+          <t>20/05/2026</t>
+        </is>
+      </c>
+      <c r="C71" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D71" s="79" t="inlineStr">
+        <is>
+          <t>SAL.vale 052026</t>
+        </is>
+      </c>
+      <c r="E71" s="79" t="inlineStr">
+        <is>
+          <t>108156/1</t>
+        </is>
+      </c>
+      <c r="F71" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G71" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H71" s="80" t="n">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B72" s="79" t="inlineStr">
+        <is>
+          <t>2026-05-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="C72" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D72" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E72" s="79" t="inlineStr">
+        <is>
+          <t>113754/5</t>
+        </is>
+      </c>
+      <c r="F72" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G72" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H72" s="80" t="n">
+        <v>207.04</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B73" s="79" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="C73" s="79" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="D73" s="79" t="inlineStr"/>
+      <c r="E73" s="79" t="inlineStr"/>
+      <c r="F73" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G73" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H73" s="80" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="79" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="B74" s="79" t="inlineStr">
+        <is>
+          <t>25/05/2026</t>
+        </is>
+      </c>
+      <c r="C74" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D74" s="79" t="inlineStr">
+        <is>
+          <t>NFS.1631</t>
+        </is>
+      </c>
+      <c r="E74" s="79" t="inlineStr">
+        <is>
+          <t>107973/1</t>
+        </is>
+      </c>
+      <c r="F74" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G74" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H74" s="80" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B75" s="79" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="C75" s="79" t="inlineStr">
+        <is>
+          <t>ALFAMA PROCESSAMENTO DE DADOS LTDA</t>
+        </is>
+      </c>
+      <c r="D75" s="79" t="inlineStr">
+        <is>
+          <t>AV.1015392</t>
+        </is>
+      </c>
+      <c r="E75" s="79" t="inlineStr">
+        <is>
+          <t>108925/1</t>
+        </is>
+      </c>
+      <c r="F75" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G75" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H75" s="80" t="n">
+        <v>183.6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B76" s="79" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="C76" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D76" s="79" t="inlineStr">
+        <is>
+          <t>FAT.21882309</t>
+        </is>
+      </c>
+      <c r="E76" s="79" t="inlineStr">
+        <is>
+          <t>111124/1</t>
+        </is>
+      </c>
+      <c r="F76" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G76" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H76" s="80" t="n">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B77" s="79" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="C77" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D77" s="79" t="inlineStr">
+        <is>
+          <t>FAT.21882309</t>
+        </is>
+      </c>
+      <c r="E77" s="79" t="inlineStr">
+        <is>
+          <t>111124/3</t>
+        </is>
+      </c>
+      <c r="F77" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G77" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H77" s="80" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B78" s="79" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="C78" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D78" s="79" t="inlineStr">
+        <is>
+          <t>NFS.373725</t>
+        </is>
+      </c>
+      <c r="E78" s="79" t="inlineStr">
+        <is>
+          <t>110785/1</t>
+        </is>
+      </c>
+      <c r="F78" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G78" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H78" s="80" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B79" s="79" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="C79" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D79" s="79" t="inlineStr">
+        <is>
+          <t>NFS.0036884701</t>
+        </is>
+      </c>
+      <c r="E79" s="79" t="inlineStr">
+        <is>
+          <t>109295/1</t>
+        </is>
+      </c>
+      <c r="F79" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G79" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H79" s="80" t="n">
+        <v>84.81999999999999</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B80" s="79" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="C80" s="79" t="inlineStr">
+        <is>
+          <t>J H ALVES - MONITOR REMOTO</t>
+        </is>
+      </c>
+      <c r="D80" s="79" t="inlineStr">
+        <is>
+          <t>NFS.78</t>
+        </is>
+      </c>
+      <c r="E80" s="79" t="inlineStr">
+        <is>
+          <t>108317/1</t>
+        </is>
+      </c>
+      <c r="F80" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G80" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H80" s="80" t="n">
+        <v>6173.37</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B81" s="79" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="C81" s="79" t="inlineStr">
+        <is>
+          <t>SABHA INTELIGENCIA EM TECNOLOGIA LTDA</t>
+        </is>
+      </c>
+      <c r="D81" s="79" t="inlineStr">
+        <is>
+          <t>NFS.5832</t>
+        </is>
+      </c>
+      <c r="E81" s="79" t="inlineStr">
+        <is>
+          <t>109227/1</t>
+        </is>
+      </c>
+      <c r="F81" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G81" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H81" s="80" t="n">
+        <v>740.38</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B82" s="79" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="C82" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D82" s="79" t="inlineStr">
+        <is>
+          <t>FAT.Vivo 04 2026</t>
+        </is>
+      </c>
+      <c r="E82" s="79" t="inlineStr">
+        <is>
+          <t>110752/1</t>
+        </is>
+      </c>
+      <c r="F82" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G82" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H82" s="80" t="n">
+        <v>184.86</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B83" s="79" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="C83" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D83" s="79" t="inlineStr">
+        <is>
+          <t>FAT.Vivo 05 2026</t>
+        </is>
+      </c>
+      <c r="E83" s="79" t="inlineStr">
+        <is>
+          <t>110753/1</t>
+        </is>
+      </c>
+      <c r="F83" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G83" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H83" s="80" t="n">
+        <v>184.86</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B84" s="79" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="C84" s="79" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D84" s="79" t="inlineStr">
+        <is>
+          <t>FAT.Vivo 06 2026</t>
+        </is>
+      </c>
+      <c r="E84" s="79" t="inlineStr">
+        <is>
+          <t>110754/1</t>
+        </is>
+      </c>
+      <c r="F84" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G84" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H84" s="80" t="n">
+        <v>184.86</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B85" s="79" t="inlineStr">
+        <is>
+          <t>15/06/2026</t>
+        </is>
+      </c>
+      <c r="C85" s="79" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="D85" s="79" t="inlineStr">
+        <is>
+          <t>BOL.1017717992</t>
+        </is>
+      </c>
+      <c r="E85" s="79" t="inlineStr">
+        <is>
+          <t>109298/1</t>
+        </is>
+      </c>
+      <c r="F85" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G85" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H85" s="80" t="n">
+        <v>137.93</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B86" s="79" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="C86" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D86" s="79" t="inlineStr">
+        <is>
+          <t>CX.27.05.26</t>
+        </is>
+      </c>
+      <c r="E86" s="79" t="inlineStr">
+        <is>
+          <t>108827/1</t>
+        </is>
+      </c>
+      <c r="F86" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G86" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H86" s="80" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B87" s="79" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="C87" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D87" s="79" t="inlineStr">
+        <is>
+          <t>SAL.1_ Ferias 1 VIn D 26</t>
+        </is>
+      </c>
+      <c r="E87" s="79" t="inlineStr">
+        <is>
+          <t>107780/1</t>
+        </is>
+      </c>
+      <c r="F87" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G87" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H87" s="80" t="n">
+        <v>1101.12</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B88" s="79" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="C88" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D88" s="79" t="inlineStr">
+        <is>
+          <t>SAL.sal 052026</t>
+        </is>
+      </c>
+      <c r="E88" s="79" t="inlineStr">
+        <is>
+          <t>109482/1</t>
+        </is>
+      </c>
+      <c r="F88" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G88" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H88" s="80" t="n">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B89" s="79" t="inlineStr">
+        <is>
+          <t>19/06/2026</t>
+        </is>
+      </c>
+      <c r="C89" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D89" s="79" t="inlineStr">
+        <is>
+          <t>SAL.SALARIO06VINI</t>
+        </is>
+      </c>
+      <c r="E89" s="79" t="inlineStr">
+        <is>
+          <t>110700/1</t>
+        </is>
+      </c>
+      <c r="F89" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G89" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H89" s="80" t="n">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B90" s="79" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="C90" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D90" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E90" s="79" t="inlineStr">
+        <is>
+          <t>113754/6</t>
+        </is>
+      </c>
+      <c r="F90" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G90" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H90" s="80" t="n">
+        <v>207.04</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B91" s="79" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="C91" s="79" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="D91" s="79" t="inlineStr"/>
+      <c r="E91" s="79" t="inlineStr"/>
+      <c r="F91" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G91" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H91" s="80" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="79" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="B92" s="79" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="C92" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D92" s="79" t="inlineStr">
+        <is>
+          <t>NFS.33</t>
+        </is>
+      </c>
+      <c r="E92" s="79" t="inlineStr">
+        <is>
+          <t>110902/1</t>
+        </is>
+      </c>
+      <c r="F92" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G92" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H92" s="80" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B93" s="79" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="C93" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D93" s="79" t="inlineStr">
+        <is>
+          <t>FAT.Claro 07.26</t>
+        </is>
+      </c>
+      <c r="E93" s="79" t="inlineStr">
+        <is>
+          <t>113575/1</t>
+        </is>
+      </c>
+      <c r="F93" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G93" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H93" s="80" t="n">
+        <v>20.39</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B94" s="79" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="C94" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D94" s="79" t="inlineStr">
+        <is>
+          <t>FAT.Claro 07.26</t>
+        </is>
+      </c>
+      <c r="E94" s="79" t="inlineStr">
+        <is>
+          <t>113575/2</t>
+        </is>
+      </c>
+      <c r="F94" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G94" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H94" s="80" t="n">
+        <v>133.73</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B95" s="79" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="C95" s="79" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="D95" s="79" t="inlineStr">
+        <is>
+          <t>FAT.Claro 07.26</t>
+        </is>
+      </c>
+      <c r="E95" s="79" t="inlineStr">
+        <is>
+          <t>113575/3</t>
+        </is>
+      </c>
+      <c r="F95" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G95" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H95" s="80" t="n">
+        <v>825.28</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B96" s="79" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="C96" s="79" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="D96" s="79" t="inlineStr">
+        <is>
+          <t>NFS.377682</t>
+        </is>
+      </c>
+      <c r="E96" s="79" t="inlineStr">
+        <is>
+          <t>114092/1</t>
+        </is>
+      </c>
+      <c r="F96" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G96" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H96" s="80" t="n">
+        <v>79.59999999999999</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B97" s="79" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="C97" s="79" t="inlineStr">
+        <is>
+          <t>J H ALVES - MONITOR REMOTO</t>
+        </is>
+      </c>
+      <c r="D97" s="79" t="inlineStr">
+        <is>
+          <t>NFS.3</t>
+        </is>
+      </c>
+      <c r="E97" s="79" t="inlineStr">
+        <is>
+          <t>111371/1</t>
+        </is>
+      </c>
+      <c r="F97" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G97" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H97" s="80" t="n">
+        <v>6300</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B98" s="79" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="C98" s="79" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="D98" s="79" t="inlineStr">
+        <is>
+          <t>BOL.LOCAWEB 07.26</t>
+        </is>
+      </c>
+      <c r="E98" s="79" t="inlineStr">
+        <is>
+          <t>113049/1</t>
+        </is>
+      </c>
+      <c r="F98" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G98" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H98" s="80" t="n">
+        <v>1151.26</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B99" s="79" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="C99" s="79" t="inlineStr">
+        <is>
+          <t>SABHA INTELIGENCIA EM TECNOLOGIA LTDA</t>
+        </is>
+      </c>
+      <c r="D99" s="79" t="inlineStr">
+        <is>
+          <t>NFS.66</t>
+        </is>
+      </c>
+      <c r="E99" s="79" t="inlineStr">
+        <is>
+          <t>112107/1</t>
+        </is>
+      </c>
+      <c r="F99" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G99" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H99" s="80" t="n">
+        <v>1037.38</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B100" s="79" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C100" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D100" s="79" t="inlineStr">
+        <is>
+          <t>SAL.sal 0626</t>
+        </is>
+      </c>
+      <c r="E100" s="79" t="inlineStr">
+        <is>
+          <t>112402/1</t>
+        </is>
+      </c>
+      <c r="F100" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G100" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H100" s="80" t="n">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B101" s="79" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="C101" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D101" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E101" s="79" t="inlineStr">
+        <is>
+          <t>113754/1</t>
+        </is>
+      </c>
+      <c r="F101" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G101" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H101" s="80" t="n">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B102" s="79" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="C102" s="79" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="D102" s="79" t="inlineStr">
+        <is>
+          <t>FGTS/INSS</t>
+        </is>
+      </c>
+      <c r="E102" s="79" t="inlineStr">
+        <is>
+          <t>113754/7</t>
+        </is>
+      </c>
+      <c r="F102" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G102" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H102" s="80" t="n">
+        <v>207.04</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B103" s="79" t="inlineStr">
+        <is>
+          <t>2026-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="C103" s="79" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="D103" s="79" t="inlineStr"/>
+      <c r="E103" s="79" t="inlineStr"/>
+      <c r="F103" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G103" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H103" s="80" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="79" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="B104" s="79" t="inlineStr">
+        <is>
+          <t>25/07/2026</t>
+        </is>
+      </c>
+      <c r="C104" s="79" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="D104" s="79" t="inlineStr">
+        <is>
+          <t>NFS.84</t>
+        </is>
+      </c>
+      <c r="E104" s="79" t="inlineStr">
+        <is>
+          <t>113583/1</t>
+        </is>
+      </c>
+      <c r="F104" s="79" t="inlineStr">
+        <is>
+          <t>Tetus</t>
+        </is>
+      </c>
+      <c r="G104" s="79" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="H104" s="80" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="G105" s="81" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="H105" s="82">
+        <f>SUM(H5:H104)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H104"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7318,4 +11397,625 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CONTAS PAGAS — RESUMO POR CREDOR  (TI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Extrato do financeiro, centro de custo "T.I". ABA DE APOIO: o centro de custo destes itens ainda não foi decidido, então nada aqui entra no Planejado, no Realizado nem no Painel. A coluna final aponta o que provavelmente já está no orçamento — confira e remova as duplicidades à mão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>Credor</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>Nº lanç.</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
+        <is>
+          <t>Jan/26</t>
+        </is>
+      </c>
+      <c r="E4" s="46" t="inlineStr">
+        <is>
+          <t>Fev/26</t>
+        </is>
+      </c>
+      <c r="F4" s="46" t="inlineStr">
+        <is>
+          <t>Mar/26</t>
+        </is>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>Abr/26</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>Mai/26</t>
+        </is>
+      </c>
+      <c r="I4" s="46" t="inlineStr">
+        <is>
+          <t>Jun/26</t>
+        </is>
+      </c>
+      <c r="J4" s="46" t="inlineStr">
+        <is>
+          <t>Jul/26</t>
+        </is>
+      </c>
+      <c r="K4" s="46" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L4" s="46" t="inlineStr">
+        <is>
+          <t>Já está no orçamento?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="56" t="inlineStr">
+        <is>
+          <t>J H ALVES - MONITOR REMOTO</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="54" t="n">
+        <v>4311.56</v>
+      </c>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n">
+        <v>3723.62</v>
+      </c>
+      <c r="I5" s="54" t="n">
+        <v>6173.37</v>
+      </c>
+      <c r="J5" s="54" t="n">
+        <v>6300</v>
+      </c>
+      <c r="K5" s="72" t="n">
+        <v>20508.55</v>
+      </c>
+      <c r="L5" s="73" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="74" t="inlineStr">
+        <is>
+          <t>VINICIUS DI FRANCO HEITOR</t>
+        </is>
+      </c>
+      <c r="B6" s="74" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C6" s="75" t="n">
+        <v>23</v>
+      </c>
+      <c r="D6" s="76" t="n">
+        <v>2670.84</v>
+      </c>
+      <c r="E6" s="76" t="n">
+        <v>2986.04</v>
+      </c>
+      <c r="F6" s="76" t="n">
+        <v>2778.04</v>
+      </c>
+      <c r="G6" s="76" t="n">
+        <v>2751.04</v>
+      </c>
+      <c r="H6" s="76" t="n">
+        <v>2719.04</v>
+      </c>
+      <c r="I6" s="76" t="n">
+        <v>3633.16</v>
+      </c>
+      <c r="J6" s="76" t="n">
+        <v>2461.04</v>
+      </c>
+      <c r="K6" s="77" t="n">
+        <v>19999.2</v>
+      </c>
+      <c r="L6" s="78" t="inlineStr">
+        <is>
+          <t>TI-E01 Vinicius Di Franco</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="74" t="inlineStr">
+        <is>
+          <t>OPENAI BRAZIL LIMITADA</t>
+        </is>
+      </c>
+      <c r="B7" s="74" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C7" s="75" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="76" t="n"/>
+      <c r="E7" s="76" t="n">
+        <v>234.46</v>
+      </c>
+      <c r="F7" s="76" t="n">
+        <v>321.76</v>
+      </c>
+      <c r="G7" s="76" t="n">
+        <v>5393.88</v>
+      </c>
+      <c r="H7" s="76" t="n"/>
+      <c r="I7" s="76" t="n"/>
+      <c r="J7" s="76" t="n"/>
+      <c r="K7" s="77" t="n">
+        <v>5950.1</v>
+      </c>
+      <c r="L7" s="78" t="inlineStr">
+        <is>
+          <t>TI-D11 GPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="56" t="inlineStr">
+        <is>
+          <t>CLARO S.A.</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>19</v>
+      </c>
+      <c r="D8" s="54" t="n">
+        <v>922.1099999999999</v>
+      </c>
+      <c r="E8" s="54" t="n"/>
+      <c r="F8" s="54" t="n">
+        <v>899.5799999999999</v>
+      </c>
+      <c r="G8" s="54" t="n">
+        <v>721.9400000000001</v>
+      </c>
+      <c r="H8" s="54" t="n">
+        <v>965.1099999999999</v>
+      </c>
+      <c r="I8" s="54" t="n">
+        <v>740</v>
+      </c>
+      <c r="J8" s="54" t="n">
+        <v>979.4</v>
+      </c>
+      <c r="K8" s="72" t="n">
+        <v>5228.139999999999</v>
+      </c>
+      <c r="L8" s="73" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="56" t="inlineStr">
+        <is>
+          <t>LOCAWEB SERVICOS DE INTERNET S/A</t>
+        </is>
+      </c>
+      <c r="B9" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C9" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="54" t="n">
+        <v>924.2800000000001</v>
+      </c>
+      <c r="E9" s="54" t="n">
+        <v>99.25</v>
+      </c>
+      <c r="F9" s="54" t="n"/>
+      <c r="G9" s="54" t="n">
+        <v>1046.52</v>
+      </c>
+      <c r="H9" s="54" t="n">
+        <v>74.81</v>
+      </c>
+      <c r="I9" s="54" t="n"/>
+      <c r="J9" s="54" t="n">
+        <v>1151.26</v>
+      </c>
+      <c r="K9" s="72" t="n">
+        <v>3296.12</v>
+      </c>
+      <c r="L9" s="73" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>SABHA INTELIGENCIA EM TECNOLOGIA LTDA</t>
+        </is>
+      </c>
+      <c r="B10" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C10" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="54" t="n">
+        <v>723.75</v>
+      </c>
+      <c r="E10" s="54" t="n"/>
+      <c r="F10" s="54" t="n"/>
+      <c r="G10" s="54" t="n"/>
+      <c r="H10" s="54" t="n">
+        <v>741.1</v>
+      </c>
+      <c r="I10" s="54" t="n">
+        <v>740.38</v>
+      </c>
+      <c r="J10" s="54" t="n">
+        <v>1037.38</v>
+      </c>
+      <c r="K10" s="72" t="n">
+        <v>3242.61</v>
+      </c>
+      <c r="L10" s="73" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="74" t="inlineStr">
+        <is>
+          <t>Vale Alimentação Vinicius</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C11" s="75" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="76" t="n"/>
+      <c r="E11" s="76" t="n">
+        <v>485</v>
+      </c>
+      <c r="F11" s="76" t="n">
+        <v>485</v>
+      </c>
+      <c r="G11" s="76" t="n">
+        <v>485</v>
+      </c>
+      <c r="H11" s="76" t="n">
+        <v>485</v>
+      </c>
+      <c r="I11" s="76" t="n">
+        <v>485</v>
+      </c>
+      <c r="J11" s="76" t="n">
+        <v>485</v>
+      </c>
+      <c r="K11" s="77" t="n">
+        <v>2910</v>
+      </c>
+      <c r="L11" s="78" t="inlineStr">
+        <is>
+          <t>TI-E01 Vinicius (benefício)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>TIM S A</t>
+        </is>
+      </c>
+      <c r="B12" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C12" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="54" t="n">
+        <v>331.42</v>
+      </c>
+      <c r="E12" s="54" t="n">
+        <v>338.5</v>
+      </c>
+      <c r="F12" s="54" t="n">
+        <v>284.63</v>
+      </c>
+      <c r="G12" s="54" t="n"/>
+      <c r="H12" s="54" t="n"/>
+      <c r="I12" s="54" t="n"/>
+      <c r="J12" s="54" t="n"/>
+      <c r="K12" s="72" t="n">
+        <v>954.5500000000001</v>
+      </c>
+      <c r="L12" s="73" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="56" t="inlineStr">
+        <is>
+          <t>VC1 SOLUCOES EM TECNOLOGIA EIRELI</t>
+        </is>
+      </c>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C13" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" s="54" t="n"/>
+      <c r="E13" s="54" t="n">
+        <v>275.84</v>
+      </c>
+      <c r="F13" s="54" t="n">
+        <v>137.9</v>
+      </c>
+      <c r="G13" s="54" t="n">
+        <v>137.9</v>
+      </c>
+      <c r="H13" s="54" t="n">
+        <v>137.92</v>
+      </c>
+      <c r="I13" s="54" t="n">
+        <v>137.93</v>
+      </c>
+      <c r="J13" s="54" t="n"/>
+      <c r="K13" s="72" t="n">
+        <v>827.49</v>
+      </c>
+      <c r="L13" s="73" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="56" t="inlineStr">
+        <is>
+          <t>TELEFONICA BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="B14" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C14" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" s="54" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="E14" s="54" t="n">
+        <v>102.32</v>
+      </c>
+      <c r="F14" s="54" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="54" t="n"/>
+      <c r="H14" s="54" t="n"/>
+      <c r="I14" s="54" t="n">
+        <v>554.58</v>
+      </c>
+      <c r="J14" s="54" t="n"/>
+      <c r="K14" s="72" t="n">
+        <v>758.53</v>
+      </c>
+      <c r="L14" s="73" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="56" t="inlineStr">
+        <is>
+          <t>WEB MOBILE TELECOM LTDA</t>
+        </is>
+      </c>
+      <c r="B15" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C15" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="E15" s="54" t="n">
+        <v>75</v>
+      </c>
+      <c r="F15" s="54" t="n">
+        <v>225</v>
+      </c>
+      <c r="G15" s="54" t="n">
+        <v>75</v>
+      </c>
+      <c r="H15" s="54" t="n">
+        <v>75</v>
+      </c>
+      <c r="I15" s="54" t="n">
+        <v>75</v>
+      </c>
+      <c r="J15" s="54" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="K15" s="72" t="n">
+        <v>690</v>
+      </c>
+      <c r="L15" s="73" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="56" t="inlineStr">
+        <is>
+          <t>INTELBRAS S.A. INDUSTRIA DE TELECOMUNICACAO ELETRONICA BRASILEIRA</t>
+        </is>
+      </c>
+      <c r="B16" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C16" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="D16" s="54" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="E16" s="54" t="n"/>
+      <c r="F16" s="54" t="n">
+        <v>159.2</v>
+      </c>
+      <c r="G16" s="54" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="H16" s="54" t="n"/>
+      <c r="I16" s="54" t="n">
+        <v>164.42</v>
+      </c>
+      <c r="J16" s="54" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="K16" s="72" t="n">
+        <v>562.42</v>
+      </c>
+      <c r="L16" s="73" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="56" t="inlineStr">
+        <is>
+          <t>ALFAMA PROCESSAMENTO DE DADOS LTDA</t>
+        </is>
+      </c>
+      <c r="B17" s="56" t="inlineStr">
+        <is>
+          <t>T.I</t>
+        </is>
+      </c>
+      <c r="C17" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="54" t="n"/>
+      <c r="E17" s="54" t="n"/>
+      <c r="F17" s="54" t="n"/>
+      <c r="G17" s="54" t="n"/>
+      <c r="H17" s="54" t="n"/>
+      <c r="I17" s="54" t="n">
+        <v>183.6</v>
+      </c>
+      <c r="J17" s="54" t="n"/>
+      <c r="K17" s="72" t="n">
+        <v>183.6</v>
+      </c>
+      <c r="L17" s="73" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="51" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="51" t="n"/>
+      <c r="C18" s="51" t="n"/>
+      <c r="D18" s="52">
+        <f>SUM(D5:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="52">
+        <f>SUM(E5:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="52">
+        <f>SUM(F5:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="52">
+        <f>SUM(G5:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="52">
+        <f>SUM(H5:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="52">
+        <f>SUM(I5:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="52">
+        <f>SUM(J5:J17)</f>
+        <v/>
+      </c>
+      <c r="K18" s="52">
+        <f>SUM(K5:K17)</f>
+        <v/>
+      </c>
+      <c r="L18" s="51" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:L17"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>